<commit_message>
Update some notes in the data extraction for women
</commit_message>
<xml_diff>
--- a/outputs/outcome_maps/women-2026-3-18T15-50.xlsx
+++ b/outputs/outcome_maps/women-2026-3-18T15-50.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddy/Library/CloudStorage/GoogleDrive-edwina.mead@monash.edu/My Drive/cost-of-excess-cs/scoping-review/public-repo/outputs/outcome_maps/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87737089-17B1-054C-A373-57B7B66C891F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{726AC18B-9AED-1D47-84D4-E63167BD118C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="pelvic floor related issues" sheetId="1" r:id="rId1"/>

</xml_diff>